<commit_message>
Updated Excel Data Day 18
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E109298A-9EEE-4A91-980C-DFE85C8CFA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9622F22-647E-4700-ACE6-53EDB916FE17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="81">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -275,6 +275,9 @@
   </si>
   <si>
     <t xml:space="preserve">I need to have better control over my emotions. </t>
+  </si>
+  <si>
+    <t>I have to leave procrastination and should focus on study more.</t>
   </si>
 </sst>
 </file>
@@ -1880,31 +1883,54 @@
         <v>79</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="str">
-        <f>IF(B23&lt;&gt;"",COUNT($B$6:B23),"")</f>
-        <v/>
-      </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="10" t="str">
+    <row r="23" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="11">
+        <v>18</v>
+      </c>
+      <c r="B23" s="8">
+        <v>46269</v>
+      </c>
+      <c r="C23" s="9">
+        <v>330</v>
+      </c>
+      <c r="D23" s="9">
+        <v>30</v>
+      </c>
+      <c r="E23" s="9">
+        <v>50</v>
+      </c>
+      <c r="F23" s="9">
+        <v>35</v>
+      </c>
+      <c r="G23" s="9">
+        <v>350</v>
+      </c>
+      <c r="H23" s="9">
+        <v>7</v>
+      </c>
+      <c r="I23" s="9">
+        <v>79</v>
+      </c>
+      <c r="J23" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K23" s="10" t="str">
+        <v>874</v>
+      </c>
+      <c r="K23" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="12"/>
+        <v>566</v>
+      </c>
+      <c r="L23" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M23" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="N23" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O23" s="12" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 19.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9622F22-647E-4700-ACE6-53EDB916FE17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21FCB173-B15D-49FF-8DF6-25E521F5C910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -278,6 +278,9 @@
   </si>
   <si>
     <t>I have to leave procrastination and should focus on study more.</t>
+  </si>
+  <si>
+    <t>Wasted my whole day doing Nothing. Need to prepare for ca.</t>
   </si>
 </sst>
 </file>
@@ -1932,31 +1935,54 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="str">
-        <f>IF(B24&lt;&gt;"",COUNT($B$6:B24),"")</f>
-        <v/>
-      </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="10" t="str">
+    <row r="24" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="11">
+        <v>19</v>
+      </c>
+      <c r="B24" s="8">
+        <v>46270</v>
+      </c>
+      <c r="C24" s="9">
+        <v>480</v>
+      </c>
+      <c r="D24" s="9">
+        <v>0</v>
+      </c>
+      <c r="E24" s="9">
+        <v>10</v>
+      </c>
+      <c r="F24" s="9">
+        <v>20</v>
+      </c>
+      <c r="G24" s="9">
+        <v>0</v>
+      </c>
+      <c r="H24" s="9">
+        <v>0</v>
+      </c>
+      <c r="I24" s="9">
+        <v>180</v>
+      </c>
+      <c r="J24" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K24" s="10" t="str">
+        <v>690</v>
+      </c>
+      <c r="K24" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="12"/>
+        <v>750</v>
+      </c>
+      <c r="L24" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M24" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N24" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O24" s="12" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 20
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21FCB173-B15D-49FF-8DF6-25E521F5C910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38B18FF-3A93-4CED-A212-276ECC7ADB53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="83">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -281,6 +281,9 @@
   </si>
   <si>
     <t>Wasted my whole day doing Nothing. Need to prepare for ca.</t>
+  </si>
+  <si>
+    <t>This will be the last day of wasting my time. From now on study.</t>
   </si>
 </sst>
 </file>
@@ -1984,31 +1987,54 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="str">
-        <f>IF(B25&lt;&gt;"",COUNT($B$6:B25),"")</f>
-        <v/>
-      </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="10" t="str">
+    <row r="25" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="11">
+        <v>20</v>
+      </c>
+      <c r="B25" s="8">
+        <v>46271</v>
+      </c>
+      <c r="C25" s="9">
+        <v>450</v>
+      </c>
+      <c r="D25" s="9">
+        <v>0</v>
+      </c>
+      <c r="E25" s="9">
+        <v>20</v>
+      </c>
+      <c r="F25" s="9">
+        <v>30</v>
+      </c>
+      <c r="G25" s="9">
+        <v>0</v>
+      </c>
+      <c r="H25" s="9">
+        <v>0</v>
+      </c>
+      <c r="I25" s="9">
+        <v>120</v>
+      </c>
+      <c r="J25" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K25" s="10" t="str">
+        <v>620</v>
+      </c>
+      <c r="K25" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="12"/>
+        <v>820</v>
+      </c>
+      <c r="L25" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M25" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="N25" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="O25" s="12" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 21
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38B18FF-3A93-4CED-A212-276ECC7ADB53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E8745C2-933A-4D47-BA6F-05CE553C2C58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -284,6 +284,9 @@
   </si>
   <si>
     <t>This will be the last day of wasting my time. From now on study.</t>
+  </si>
+  <si>
+    <t>Others are doing so much and here I am doing nothing but that will change.</t>
   </si>
 </sst>
 </file>
@@ -2036,31 +2039,54 @@
         <v>82</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="str">
-        <f>IF(B26&lt;&gt;"",COUNT($B$6:B26),"")</f>
-        <v/>
-      </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="10" t="str">
+    <row r="26" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="11">
+        <v>21</v>
+      </c>
+      <c r="B26" s="8">
+        <v>46272</v>
+      </c>
+      <c r="C26" s="9">
+        <v>330</v>
+      </c>
+      <c r="D26" s="9">
+        <v>20</v>
+      </c>
+      <c r="E26" s="9">
+        <v>40</v>
+      </c>
+      <c r="F26" s="9">
+        <v>40</v>
+      </c>
+      <c r="G26" s="9">
+        <v>300</v>
+      </c>
+      <c r="H26" s="9">
+        <v>5</v>
+      </c>
+      <c r="I26" s="9">
+        <v>80</v>
+      </c>
+      <c r="J26" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K26" s="10" t="str">
+        <v>810</v>
+      </c>
+      <c r="K26" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
-      <c r="N26" s="11"/>
-      <c r="O26" s="12"/>
+        <v>630</v>
+      </c>
+      <c r="L26" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="M26" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N26" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O26" s="12" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 22
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E8745C2-933A-4D47-BA6F-05CE553C2C58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B0ED43A-6319-4008-B380-6F8756E222A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="85">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -287,6 +287,9 @@
   </si>
   <si>
     <t>Others are doing so much and here I am doing nothing but that will change.</t>
+  </si>
+  <si>
+    <t>I couldn't perform well in my communication presentation.</t>
   </si>
 </sst>
 </file>
@@ -2088,31 +2091,54 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A27" s="11" t="str">
-        <f>IF(B27&lt;&gt;"",COUNT($B$6:B27),"")</f>
-        <v/>
-      </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="10" t="str">
+    <row r="27" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="11">
+        <v>22</v>
+      </c>
+      <c r="B27" s="8">
+        <v>46273</v>
+      </c>
+      <c r="C27" s="9">
+        <v>360</v>
+      </c>
+      <c r="D27" s="9">
+        <v>30</v>
+      </c>
+      <c r="E27" s="9">
+        <v>50</v>
+      </c>
+      <c r="F27" s="9">
+        <v>50</v>
+      </c>
+      <c r="G27" s="9">
+        <v>300</v>
+      </c>
+      <c r="H27" s="9">
+        <v>5</v>
+      </c>
+      <c r="I27" s="9">
+        <v>240</v>
+      </c>
+      <c r="J27" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K27" s="10" t="str">
+        <v>1030</v>
+      </c>
+      <c r="K27" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
-      <c r="N27" s="11"/>
-      <c r="O27" s="12"/>
+        <v>410</v>
+      </c>
+      <c r="L27" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M27" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="N27" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O27" s="12" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 23.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B0ED43A-6319-4008-B380-6F8756E222A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F83FBACE-F662-4C18-A331-73BC66073161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="86">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -290,6 +290,9 @@
   </si>
   <si>
     <t>I couldn't perform well in my communication presentation.</t>
+  </si>
+  <si>
+    <t>I think I did good in my dbms CA.</t>
   </si>
 </sst>
 </file>
@@ -2141,30 +2144,53 @@
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="str">
-        <f>IF(B28&lt;&gt;"",COUNT($B$6:B28),"")</f>
-        <v/>
-      </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="10" t="str">
+      <c r="A28" s="11">
+        <v>23</v>
+      </c>
+      <c r="B28" s="8">
+        <v>46274</v>
+      </c>
+      <c r="C28" s="9">
+        <v>350</v>
+      </c>
+      <c r="D28" s="9">
+        <v>20</v>
+      </c>
+      <c r="E28" s="9">
+        <v>40</v>
+      </c>
+      <c r="F28" s="9">
+        <v>60</v>
+      </c>
+      <c r="G28" s="9">
+        <v>300</v>
+      </c>
+      <c r="H28" s="9">
+        <v>5</v>
+      </c>
+      <c r="I28" s="9">
+        <v>60</v>
+      </c>
+      <c r="J28" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K28" s="10" t="str">
+        <v>830</v>
+      </c>
+      <c r="K28" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="11"/>
-      <c r="O28" s="12"/>
+        <v>610</v>
+      </c>
+      <c r="L28" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M28" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="N28" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="O28" s="12" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 24.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F83FBACE-F662-4C18-A331-73BC66073161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0526D0C7-AEB9-482E-8A0F-29CDF8DDA031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="87">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -293,6 +293,9 @@
   </si>
   <si>
     <t>I think I did good in my dbms CA.</t>
+  </si>
+  <si>
+    <t>Today was fresher's day. I realized I am not a fan of these type of things.</t>
   </si>
 </sst>
 </file>
@@ -2192,31 +2195,54 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A29" s="11" t="str">
-        <f>IF(B29&lt;&gt;"",COUNT($B$6:B29),"")</f>
-        <v/>
-      </c>
-      <c r="B29" s="8"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="10" t="str">
+    <row r="29" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="11">
+        <v>24</v>
+      </c>
+      <c r="B29" s="8">
+        <v>46275</v>
+      </c>
+      <c r="C29" s="9">
+        <v>380</v>
+      </c>
+      <c r="D29" s="9">
+        <v>30</v>
+      </c>
+      <c r="E29" s="9">
+        <v>80</v>
+      </c>
+      <c r="F29" s="9">
+        <v>10</v>
+      </c>
+      <c r="G29" s="9">
+        <v>100</v>
+      </c>
+      <c r="H29" s="9">
+        <v>2</v>
+      </c>
+      <c r="I29" s="9">
+        <v>15</v>
+      </c>
+      <c r="J29" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K29" s="10" t="str">
+        <v>615</v>
+      </c>
+      <c r="K29" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
-      <c r="N29" s="11"/>
-      <c r="O29" s="12"/>
+        <v>825</v>
+      </c>
+      <c r="L29" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M29" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N29" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O29" s="12" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel File Day 25.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0526D0C7-AEB9-482E-8A0F-29CDF8DDA031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E71E61F-9094-4637-B104-5F22AA237119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="88">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -296,6 +296,9 @@
   </si>
   <si>
     <t>Today was fresher's day. I realized I am not a fan of these type of things.</t>
+  </si>
+  <si>
+    <t>Need to prepare for Analytical Skills upcoming CA exams.</t>
   </si>
 </sst>
 </file>
@@ -2244,31 +2247,54 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A30" s="11" t="str">
-        <f>IF(B30&lt;&gt;"",COUNT($B$6:B30),"")</f>
-        <v/>
-      </c>
-      <c r="B30" s="8"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="10" t="str">
+    <row r="30" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="11">
+        <v>25</v>
+      </c>
+      <c r="B30" s="8">
+        <v>46276</v>
+      </c>
+      <c r="C30" s="9">
+        <v>410</v>
+      </c>
+      <c r="D30" s="9">
+        <v>20</v>
+      </c>
+      <c r="E30" s="9">
+        <v>40</v>
+      </c>
+      <c r="F30" s="9">
+        <v>50</v>
+      </c>
+      <c r="G30" s="9">
+        <v>300</v>
+      </c>
+      <c r="H30" s="9">
+        <v>6</v>
+      </c>
+      <c r="I30" s="9">
+        <v>60</v>
+      </c>
+      <c r="J30" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K30" s="10" t="str">
+        <v>880</v>
+      </c>
+      <c r="K30" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
-      <c r="N30" s="11"/>
-      <c r="O30" s="12"/>
+        <v>560</v>
+      </c>
+      <c r="L30" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M30" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="N30" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O30" s="12" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 26.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E71E61F-9094-4637-B104-5F22AA237119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FCFFD0F-074F-4DBD-A392-1E031C43AAC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -299,6 +299,9 @@
   </si>
   <si>
     <t>Need to prepare for Analytical Skills upcoming CA exams.</t>
+  </si>
+  <si>
+    <t>Sometimes all you need is just a break from everything.</t>
   </si>
 </sst>
 </file>
@@ -2296,31 +2299,54 @@
         <v>87</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A31" s="11" t="str">
-        <f>IF(B31&lt;&gt;"",COUNT($B$6:B31),"")</f>
-        <v/>
-      </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="10" t="str">
+    <row r="31" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="11">
+        <v>26</v>
+      </c>
+      <c r="B31" s="8">
+        <v>46277</v>
+      </c>
+      <c r="C31" s="9">
+        <v>450</v>
+      </c>
+      <c r="D31" s="9">
+        <v>10</v>
+      </c>
+      <c r="E31" s="9">
+        <v>15</v>
+      </c>
+      <c r="F31" s="9">
+        <v>30</v>
+      </c>
+      <c r="G31" s="9">
+        <v>0</v>
+      </c>
+      <c r="H31" s="9">
+        <v>0</v>
+      </c>
+      <c r="I31" s="9">
+        <v>240</v>
+      </c>
+      <c r="J31" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K31" s="10" t="str">
+        <v>745</v>
+      </c>
+      <c r="K31" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="N31" s="11"/>
-      <c r="O31" s="12"/>
+        <v>695</v>
+      </c>
+      <c r="L31" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M31" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="N31" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="O31" s="12" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 27.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FCFFD0F-074F-4DBD-A392-1E031C43AAC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4C5DEE-1864-42C1-BF90-83EF645A90F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t>Sometimes all you need is just a break from everything.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today I did nothing productive. </t>
   </si>
 </sst>
 </file>
@@ -2349,30 +2352,53 @@
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A32" s="11" t="str">
-        <f>IF(B32&lt;&gt;"",COUNT($B$6:B32),"")</f>
-        <v/>
-      </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="9"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="9"/>
-      <c r="H32" s="9"/>
-      <c r="I32" s="9"/>
-      <c r="J32" s="10" t="str">
+      <c r="A32" s="11">
+        <v>27</v>
+      </c>
+      <c r="B32" s="8">
+        <v>46278</v>
+      </c>
+      <c r="C32" s="9">
+        <v>300</v>
+      </c>
+      <c r="D32" s="9">
+        <v>0</v>
+      </c>
+      <c r="E32" s="9">
+        <v>20</v>
+      </c>
+      <c r="F32" s="9">
+        <v>50</v>
+      </c>
+      <c r="G32" s="9">
+        <v>0</v>
+      </c>
+      <c r="H32" s="9">
+        <v>0</v>
+      </c>
+      <c r="I32" s="9">
+        <v>300</v>
+      </c>
+      <c r="J32" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K32" s="10" t="str">
+        <v>670</v>
+      </c>
+      <c r="K32" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="11"/>
-      <c r="O32" s="12"/>
+        <v>770</v>
+      </c>
+      <c r="L32" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M32" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="N32" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O32" s="12" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 28,29.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4C5DEE-1864-42C1-BF90-83EF645A90F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{210904A1-D523-428D-925B-D00BCF1A12E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="94">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -305,6 +305,18 @@
   </si>
   <si>
     <t xml:space="preserve">Today I did nothing productive. </t>
+  </si>
+  <si>
+    <t>Today I gave mars test. I need to better in python.</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Today I went with my friend. Being with them makes me happy.</t>
   </si>
 </sst>
 </file>
@@ -2400,63 +2412,106 @@
         <v>89</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A33" s="11" t="str">
-        <f>IF(B33&lt;&gt;"",COUNT($B$6:B33),"")</f>
-        <v/>
-      </c>
-      <c r="B33" s="8"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="9"/>
-      <c r="H33" s="9"/>
-      <c r="I33" s="9"/>
-      <c r="J33" s="10" t="str">
+    <row r="33" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="11">
+        <v>28</v>
+      </c>
+      <c r="B33" s="8">
+        <v>46279</v>
+      </c>
+      <c r="C33" s="9">
+        <v>420</v>
+      </c>
+      <c r="D33" s="9">
+        <v>15</v>
+      </c>
+      <c r="E33" s="9">
+        <v>40</v>
+      </c>
+      <c r="F33" s="9">
+        <v>60</v>
+      </c>
+      <c r="G33" s="9">
+        <v>200</v>
+      </c>
+      <c r="H33" s="9">
+        <v>4</v>
+      </c>
+      <c r="I33" s="9">
+        <v>200</v>
+      </c>
+      <c r="J33" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K33" s="10" t="str">
+        <v>935</v>
+      </c>
+      <c r="K33" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
-      <c r="N33" s="11"/>
-      <c r="O33" s="12"/>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A34" s="11" t="str">
-        <f>IF(B34&lt;&gt;"",COUNT($B$6:B34),"")</f>
-        <v/>
-      </c>
-      <c r="B34" s="8"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="10" t="str">
+        <v>505</v>
+      </c>
+      <c r="L33" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="N33" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O33" s="12" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="11">
+        <v>29</v>
+      </c>
+      <c r="B34" s="8">
+        <v>46280</v>
+      </c>
+      <c r="C34" s="9">
+        <v>330</v>
+      </c>
+      <c r="D34" s="9">
+        <v>10</v>
+      </c>
+      <c r="E34" s="9">
+        <v>20</v>
+      </c>
+      <c r="F34" s="9">
+        <v>40</v>
+      </c>
+      <c r="G34" s="9">
+        <v>250</v>
+      </c>
+      <c r="H34" s="9">
+        <v>5</v>
+      </c>
+      <c r="I34" s="9">
+        <v>150</v>
+      </c>
+      <c r="J34" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K34" s="10" t="str">
+        <v>800</v>
+      </c>
+      <c r="K34" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L34" s="11"/>
-      <c r="M34" s="11"/>
-      <c r="N34" s="11"/>
-      <c r="O34" s="12"/>
+        <v>640</v>
+      </c>
+      <c r="L34" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M34" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N34" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O34" s="12" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="11" t="str">
-        <f>IF(B35&lt;&gt;"",COUNT($B$6:B35),"")</f>
-        <v/>
-      </c>
+      <c r="A35" s="11"/>
       <c r="B35" s="8"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>

</xml_diff>

<commit_message>
Updated Excel Data Day 30.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{210904A1-D523-428D-925B-D00BCF1A12E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13CA8BED-D707-4F53-9BE9-B82844DBFC6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="95">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -304,19 +304,22 @@
     <t>Sometimes all you need is just a break from everything.</t>
   </si>
   <si>
-    <t xml:space="preserve">Today I did nothing productive. </t>
-  </si>
-  <si>
-    <t>Today I gave mars test. I need to better in python.</t>
-  </si>
-  <si>
     <t>Excellent</t>
   </si>
   <si>
     <t>Very Satisfied</t>
   </si>
   <si>
-    <t>Today I went with my friend. Being with them makes me happy.</t>
+    <t>Today I gave mars test. I need to do better in python.</t>
+  </si>
+  <si>
+    <t>Today I did nothing productive and just wasted my day.</t>
+  </si>
+  <si>
+    <t>I should have better control on my emotions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analytical Skills test date has been out. </t>
   </si>
 </sst>
 </file>
@@ -2363,7 +2366,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="11">
         <v>27</v>
       </c>
@@ -2409,10 +2412,10 @@
         <v>51</v>
       </c>
       <c r="O32" s="12" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="11">
         <v>28</v>
       </c>
@@ -2449,10 +2452,10 @@
         <v>505</v>
       </c>
       <c r="L33" s="11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="M33" s="11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="N33" s="11" t="s">
         <v>51</v>
@@ -2507,31 +2510,57 @@
         <v>51</v>
       </c>
       <c r="O34" s="12" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="11">
+        <v>30</v>
+      </c>
+      <c r="B35" s="8">
+        <v>46281</v>
+      </c>
+      <c r="C35" s="9">
+        <v>510</v>
+      </c>
+      <c r="D35" s="9">
+        <v>0</v>
+      </c>
+      <c r="E35" s="9">
+        <v>60</v>
+      </c>
+      <c r="F35" s="9">
+        <v>30</v>
+      </c>
+      <c r="G35" s="9">
+        <v>250</v>
+      </c>
+      <c r="H35" s="9">
+        <v>5</v>
+      </c>
+      <c r="I35" s="9">
         <v>90</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="11"/>
-      <c r="B35" s="8"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="10" t="str">
+      <c r="J35" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K35" s="10" t="str">
+        <v>940</v>
+      </c>
+      <c r="K35" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L35" s="11"/>
-      <c r="M35" s="11"/>
-      <c r="N35" s="11"/>
-      <c r="O35" s="12"/>
+        <v>500</v>
+      </c>
+      <c r="L35" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M35" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N35" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O35" s="12" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 31.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13CA8BED-D707-4F53-9BE9-B82844DBFC6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9E1A50-F0B4-4C2C-B619-C110EF447C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="96">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -320,6 +320,9 @@
   </si>
   <si>
     <t xml:space="preserve">Analytical Skills test date has been out. </t>
+  </si>
+  <si>
+    <t>Feeling stressed I don't know how I would be able to do better.</t>
   </si>
 </sst>
 </file>
@@ -2562,31 +2565,54 @@
         <v>94</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A36" s="11" t="str">
-        <f>IF(B36&lt;&gt;"",COUNT($B$6:B36),"")</f>
-        <v/>
-      </c>
-      <c r="B36" s="8"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="9"/>
-      <c r="J36" s="10" t="str">
+    <row r="36" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A36" s="11">
+        <v>31</v>
+      </c>
+      <c r="B36" s="8">
+        <v>46282</v>
+      </c>
+      <c r="C36" s="9">
+        <v>290</v>
+      </c>
+      <c r="D36" s="9">
+        <v>10</v>
+      </c>
+      <c r="E36" s="9">
+        <v>45</v>
+      </c>
+      <c r="F36" s="9">
+        <v>30</v>
+      </c>
+      <c r="G36" s="9">
+        <v>300</v>
+      </c>
+      <c r="H36" s="9">
+        <v>6</v>
+      </c>
+      <c r="I36" s="9">
+        <v>60</v>
+      </c>
+      <c r="J36" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K36" s="10" t="str">
+        <v>735</v>
+      </c>
+      <c r="K36" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L36" s="11"/>
-      <c r="M36" s="11"/>
-      <c r="N36" s="11"/>
-      <c r="O36" s="12"/>
+        <v>705</v>
+      </c>
+      <c r="L36" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M36" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N36" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O36" s="12" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 32.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9E1A50-F0B4-4C2C-B619-C110EF447C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35AD2FD-EC17-40A8-8F85-495063DEA434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="97">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -323,6 +323,9 @@
   </si>
   <si>
     <t>Feeling stressed I don't know how I would be able to do better.</t>
+  </si>
+  <si>
+    <t>Solving Analytical Problems for two period is very exhausting.</t>
   </si>
 </sst>
 </file>
@@ -2614,37 +2617,57 @@
         <v>95</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A37" s="11" t="str">
-        <f>IF(B37&lt;&gt;"",COUNT($B$6:B37),"")</f>
-        <v/>
-      </c>
-      <c r="B37" s="8"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="9"/>
-      <c r="H37" s="9"/>
-      <c r="I37" s="9"/>
-      <c r="J37" s="10" t="str">
+    <row r="37" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="11">
+        <v>32</v>
+      </c>
+      <c r="B37" s="8">
+        <v>46283</v>
+      </c>
+      <c r="C37" s="9">
+        <v>350</v>
+      </c>
+      <c r="D37" s="9">
+        <v>15</v>
+      </c>
+      <c r="E37" s="9">
+        <v>40</v>
+      </c>
+      <c r="F37" s="9">
+        <v>45</v>
+      </c>
+      <c r="G37" s="9">
+        <v>350</v>
+      </c>
+      <c r="H37" s="9">
+        <v>7</v>
+      </c>
+      <c r="I37" s="9">
+        <v>90</v>
+      </c>
+      <c r="J37" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K37" s="10" t="str">
+        <v>890</v>
+      </c>
+      <c r="K37" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L37" s="11"/>
-      <c r="M37" s="11"/>
-      <c r="N37" s="11"/>
-      <c r="O37" s="12"/>
+        <v>550</v>
+      </c>
+      <c r="L37" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M37" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="N37" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O37" s="12" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="11" t="str">
-        <f>IF(B38&lt;&gt;"",COUNT($B$6:B38),"")</f>
-        <v/>
-      </c>
+      <c r="A38" s="11"/>
       <c r="B38" s="8"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>

</xml_diff>

<commit_message>
Updated Excel Data Day 33.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35AD2FD-EC17-40A8-8F85-495063DEA434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA59C740-1C09-4EB7-B8B0-630678AF74F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="98">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -326,6 +326,9 @@
   </si>
   <si>
     <t>Solving Analytical Problems for two period is very exhausting.</t>
+  </si>
+  <si>
+    <t>Why do LPU held CA's exams online if they can't manage to do that properly. They have ruined my whole day.</t>
   </si>
 </sst>
 </file>
@@ -2666,28 +2669,54 @@
         <v>96</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="11"/>
-      <c r="B38" s="8"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="9"/>
-      <c r="I38" s="9"/>
-      <c r="J38" s="10" t="str">
+    <row r="38" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="11">
+        <v>33</v>
+      </c>
+      <c r="B38" s="8">
+        <v>46284</v>
+      </c>
+      <c r="C38" s="9">
+        <v>240</v>
+      </c>
+      <c r="D38" s="9">
+        <v>10</v>
+      </c>
+      <c r="E38" s="9">
+        <v>20</v>
+      </c>
+      <c r="F38" s="9">
+        <v>10</v>
+      </c>
+      <c r="G38" s="9">
+        <v>60</v>
+      </c>
+      <c r="H38" s="9">
+        <v>1</v>
+      </c>
+      <c r="I38" s="9">
+        <v>360</v>
+      </c>
+      <c r="J38" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K38" s="10" t="str">
+        <v>700</v>
+      </c>
+      <c r="K38" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L38" s="11"/>
-      <c r="M38" s="11"/>
-      <c r="N38" s="11"/>
-      <c r="O38" s="12"/>
+        <v>740</v>
+      </c>
+      <c r="L38" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="M38" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="N38" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O38" s="12" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 41.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26FF66F9-BD7E-4B69-8968-8D629ACB22A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1CCF60-735B-4513-A234-537012330A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="105">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -348,6 +348,9 @@
   <si>
     <t>I was having a bad day and I even scored badly in one of my CA's</t>
   </si>
+  <si>
+    <t>Working on python minor project and researching.</t>
+  </si>
 </sst>
 </file>
 
@@ -557,7 +560,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -570,51 +572,16 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1093,74 +1060,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>53</v>
       </c>
       <c r="C2" s="20"/>
-      <c r="D2" s="19"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="19">
         <v>12612197</v>
       </c>
-      <c r="G2" s="19"/>
+      <c r="G2" s="21"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>54</v>
       </c>
       <c r="C3" s="20"/>
-      <c r="D3" s="19"/>
+      <c r="D3" s="21"/>
       <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="21"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="17"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="17"/>
     </row>
     <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -1207,1866 +1174,1890 @@
       </c>
     </row>
     <row r="6" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="14">
+      <c r="A6" s="13">
         <v>46247</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="14">
         <v>450</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="14">
         <v>20</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="14">
         <v>30</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="14">
         <v>0</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="14">
         <v>300</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="14">
         <v>6</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H6" s="14">
         <v>240</v>
       </c>
-      <c r="I6" s="16">
+      <c r="I6" s="15">
         <f t="shared" ref="I6:I69" si="0">IF(SUM(B6:F6,H6)=0,"",SUM(B6:F6,H6))</f>
         <v>1040</v>
       </c>
-      <c r="J6" s="16">
+      <c r="J6" s="15">
         <f t="shared" ref="J6:J69" si="1">IF(I6="","",1440-I6)</f>
         <v>400</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L6" s="17" t="s">
+      <c r="L6" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M6" s="17" t="s">
+      <c r="M6" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="N6" s="17" t="s">
+      <c r="N6" s="16" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="14">
+      <c r="A7" s="13">
         <v>46248</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="14">
         <v>360</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="14">
         <v>15</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="14">
         <v>20</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="14">
         <v>25</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="14">
         <v>350</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="14">
         <v>7</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="14">
         <v>180</v>
       </c>
-      <c r="I7" s="16">
+      <c r="I7" s="15">
         <f t="shared" si="0"/>
         <v>950</v>
       </c>
-      <c r="J7" s="16">
+      <c r="J7" s="15">
         <f t="shared" si="1"/>
         <v>490</v>
       </c>
-      <c r="K7" s="17" t="s">
+      <c r="K7" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L7" s="17" t="s">
+      <c r="L7" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M7" s="17" t="s">
+      <c r="M7" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N7" s="17" t="s">
+      <c r="N7" s="16" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="14">
+      <c r="A8" s="13">
         <v>46249</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="14">
         <v>510</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="14">
         <v>0</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="14">
         <v>40</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="14">
         <v>60</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="14">
         <v>0</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="14">
         <v>0</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8" s="14">
         <v>150</v>
       </c>
-      <c r="I8" s="16">
+      <c r="I8" s="15">
         <f t="shared" si="0"/>
         <v>760</v>
       </c>
-      <c r="J8" s="16">
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
         <v>680</v>
       </c>
-      <c r="K8" s="17" t="s">
+      <c r="K8" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L8" s="17" t="s">
+      <c r="L8" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M8" s="17" t="s">
+      <c r="M8" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N8" s="17" t="s">
+      <c r="N8" s="16" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="14">
+      <c r="A9" s="13">
         <v>46250</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="14">
         <v>450</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="14">
         <v>10</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="14">
         <v>35</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="14">
         <v>45</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="14">
         <v>0</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="14">
         <v>0</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="14">
         <v>90</v>
       </c>
-      <c r="I9" s="16">
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
         <v>630</v>
       </c>
-      <c r="J9" s="16">
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
         <v>810</v>
       </c>
-      <c r="K9" s="17" t="s">
+      <c r="K9" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L9" s="17" t="s">
+      <c r="L9" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="M9" s="17" t="s">
+      <c r="M9" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N9" s="17" t="s">
+      <c r="N9" s="16" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="14">
+      <c r="A10" s="13">
         <v>46251</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="14">
         <v>380</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="14">
         <v>30</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="14">
         <v>20</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="14">
         <v>40</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="14">
         <v>200</v>
       </c>
-      <c r="G10" s="15">
+      <c r="G10" s="14">
         <v>4</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="14">
         <v>210</v>
       </c>
-      <c r="I10" s="16">
+      <c r="I10" s="15">
         <f t="shared" si="0"/>
         <v>880</v>
       </c>
-      <c r="J10" s="16">
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
         <v>560</v>
       </c>
-      <c r="K10" s="17" t="s">
+      <c r="K10" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L10" s="17" t="s">
+      <c r="L10" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M10" s="17" t="s">
+      <c r="M10" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N10" s="17" t="s">
+      <c r="N10" s="16" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="14">
+      <c r="A11" s="13">
         <v>46252</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="14">
         <v>320</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="14">
         <v>5</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="14">
         <v>28</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="14">
         <v>17</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="14">
         <v>300</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G11" s="14">
         <v>6</v>
       </c>
-      <c r="H11" s="15">
+      <c r="H11" s="14">
         <v>45</v>
       </c>
-      <c r="I11" s="16">
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
         <v>715</v>
       </c>
-      <c r="J11" s="16">
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
         <v>725</v>
       </c>
-      <c r="K11" s="17" t="s">
+      <c r="K11" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L11" s="17" t="s">
+      <c r="L11" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M11" s="17" t="s">
+      <c r="M11" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N11" s="17" t="s">
+      <c r="N11" s="16" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="14">
+      <c r="A12" s="13">
         <v>46253</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="14">
         <v>390</v>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="14">
         <v>18</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="14">
         <v>25</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="14">
         <v>70</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="14">
         <v>350</v>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="14">
         <v>7</v>
       </c>
-      <c r="H12" s="15">
+      <c r="H12" s="14">
         <v>60</v>
       </c>
-      <c r="I12" s="16">
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
         <v>913</v>
       </c>
-      <c r="J12" s="16">
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
         <v>527</v>
       </c>
-      <c r="K12" s="17" t="s">
+      <c r="K12" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L12" s="17" t="s">
+      <c r="L12" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M12" s="17" t="s">
+      <c r="M12" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N12" s="17" t="s">
+      <c r="N12" s="16" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="14">
+      <c r="A13" s="13">
         <v>46254</v>
       </c>
-      <c r="B13" s="15">
+      <c r="B13" s="14">
         <v>370</v>
       </c>
-      <c r="C13" s="15">
+      <c r="C13" s="14">
         <v>45</v>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="14">
         <v>40</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="14">
         <v>55</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="14">
         <v>150</v>
       </c>
-      <c r="G13" s="15">
+      <c r="G13" s="14">
         <v>3</v>
       </c>
-      <c r="H13" s="15">
+      <c r="H13" s="14">
         <v>55</v>
       </c>
-      <c r="I13" s="16">
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
         <v>715</v>
       </c>
-      <c r="J13" s="16">
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
         <v>725</v>
       </c>
-      <c r="K13" s="17" t="s">
+      <c r="K13" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L13" s="17" t="s">
+      <c r="L13" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M13" s="17" t="s">
+      <c r="M13" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N13" s="17" t="s">
+      <c r="N13" s="16" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="14">
+      <c r="A14" s="13">
         <v>46255</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="14">
         <v>440</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="14">
         <v>15</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="14">
         <v>70</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="14">
         <v>95</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="14">
         <v>0</v>
       </c>
-      <c r="G14" s="15">
+      <c r="G14" s="14">
         <v>0</v>
       </c>
-      <c r="H14" s="15">
+      <c r="H14" s="14">
         <v>120</v>
       </c>
-      <c r="I14" s="16">
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
         <v>740</v>
       </c>
-      <c r="J14" s="16">
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
         <v>700</v>
       </c>
-      <c r="K14" s="17" t="s">
+      <c r="K14" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L14" s="17" t="s">
+      <c r="L14" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M14" s="17" t="s">
+      <c r="M14" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N14" s="17" t="s">
+      <c r="N14" s="16" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="14">
+      <c r="A15" s="13">
         <v>46256</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="14">
         <v>510</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="14">
         <v>0</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="14">
         <v>35</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="14">
         <v>30</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="14">
         <v>0</v>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="14">
         <v>0</v>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="14">
         <v>155</v>
       </c>
-      <c r="I15" s="16">
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
         <v>730</v>
       </c>
-      <c r="J15" s="16">
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
         <v>710</v>
       </c>
-      <c r="K15" s="17" t="s">
+      <c r="K15" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L15" s="17" t="s">
+      <c r="L15" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M15" s="17" t="s">
+      <c r="M15" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N15" s="17" t="s">
+      <c r="N15" s="16" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="14">
+      <c r="A16" s="13">
         <v>46257</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="14">
         <v>540</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="14">
         <v>20</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="14">
         <v>80</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="14">
         <v>100</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="14">
         <v>0</v>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="14">
         <v>0</v>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="14">
         <v>90</v>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
         <v>830</v>
       </c>
-      <c r="J16" s="16">
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
         <v>610</v>
       </c>
-      <c r="K16" s="17" t="s">
+      <c r="K16" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L16" s="17" t="s">
+      <c r="L16" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M16" s="17" t="s">
+      <c r="M16" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="N16" s="17" t="s">
+      <c r="N16" s="16" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="14">
+      <c r="A17" s="13">
         <v>46258</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="14">
         <v>370</v>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="14">
         <v>10</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="14">
         <v>20</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="14">
         <v>60</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="14">
         <v>200</v>
       </c>
-      <c r="G17" s="15">
+      <c r="G17" s="14">
         <v>4</v>
       </c>
-      <c r="H17" s="15">
+      <c r="H17" s="14">
         <v>80</v>
       </c>
-      <c r="I17" s="16">
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
         <v>740</v>
       </c>
-      <c r="J17" s="16">
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
         <v>700</v>
       </c>
-      <c r="K17" s="17" t="s">
+      <c r="K17" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L17" s="17" t="s">
+      <c r="L17" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M17" s="17" t="s">
+      <c r="M17" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N17" s="17" t="s">
+      <c r="N17" s="16" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A18" s="14">
+      <c r="A18" s="13">
         <v>46259</v>
       </c>
-      <c r="B18" s="15">
+      <c r="B18" s="14">
         <v>360</v>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="14">
         <v>20</v>
       </c>
-      <c r="D18" s="15">
+      <c r="D18" s="14">
         <v>40</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="14">
         <v>50</v>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="14">
         <v>250</v>
       </c>
-      <c r="G18" s="15">
+      <c r="G18" s="14">
         <v>5</v>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="14">
         <v>90</v>
       </c>
-      <c r="I18" s="16">
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
         <v>810</v>
       </c>
-      <c r="J18" s="16">
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
         <v>630</v>
       </c>
-      <c r="K18" s="17" t="s">
+      <c r="K18" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L18" s="17" t="s">
+      <c r="L18" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M18" s="17" t="s">
+      <c r="M18" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N18" s="17" t="s">
+      <c r="N18" s="16" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="14">
+      <c r="A19" s="13">
         <v>46260</v>
       </c>
-      <c r="B19" s="15">
+      <c r="B19" s="14">
         <v>330</v>
       </c>
-      <c r="C19" s="15">
+      <c r="C19" s="14">
         <v>30</v>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="14">
         <v>50</v>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="14">
         <v>120</v>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="14">
         <v>250</v>
       </c>
-      <c r="G19" s="15">
+      <c r="G19" s="14">
         <v>5</v>
       </c>
-      <c r="H19" s="15">
+      <c r="H19" s="14">
         <v>10</v>
       </c>
-      <c r="I19" s="16">
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
         <v>790</v>
       </c>
-      <c r="J19" s="16">
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
         <v>650</v>
       </c>
-      <c r="K19" s="17" t="s">
+      <c r="K19" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L19" s="17" t="s">
+      <c r="L19" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M19" s="17" t="s">
+      <c r="M19" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N19" s="17" t="s">
+      <c r="N19" s="16" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="14">
+      <c r="A20" s="13">
         <v>46261</v>
       </c>
-      <c r="B20" s="15">
+      <c r="B20" s="14">
         <v>500</v>
       </c>
-      <c r="C20" s="15">
+      <c r="C20" s="14">
         <v>20</v>
       </c>
-      <c r="D20" s="15">
+      <c r="D20" s="14">
         <v>30</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="14">
         <v>120</v>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="14">
         <v>300</v>
       </c>
-      <c r="G20" s="15">
+      <c r="G20" s="14">
         <v>6</v>
       </c>
-      <c r="H20" s="15">
+      <c r="H20" s="14">
         <v>50</v>
       </c>
-      <c r="I20" s="16">
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
         <v>1020</v>
       </c>
-      <c r="J20" s="16">
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
         <v>420</v>
       </c>
-      <c r="K20" s="17" t="s">
+      <c r="K20" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L20" s="17" t="s">
+      <c r="L20" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M20" s="17" t="s">
+      <c r="M20" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N20" s="17" t="s">
+      <c r="N20" s="16" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="14">
+      <c r="A21" s="13">
         <v>46262</v>
       </c>
-      <c r="B21" s="15">
+      <c r="B21" s="14">
         <v>345</v>
       </c>
-      <c r="C21" s="15">
+      <c r="C21" s="14">
         <v>25</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="14">
         <v>45</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="14">
         <v>65</v>
       </c>
-      <c r="F21" s="15">
+      <c r="F21" s="14">
         <v>200</v>
       </c>
-      <c r="G21" s="15">
+      <c r="G21" s="14">
         <v>4</v>
       </c>
-      <c r="H21" s="15">
+      <c r="H21" s="14">
         <v>30</v>
       </c>
-      <c r="I21" s="16">
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
         <v>710</v>
       </c>
-      <c r="J21" s="16">
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
         <v>730</v>
       </c>
-      <c r="K21" s="17" t="s">
+      <c r="K21" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="L21" s="17" t="s">
+      <c r="L21" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="M21" s="17" t="s">
+      <c r="M21" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N21" s="17" t="s">
+      <c r="N21" s="16" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="14">
+      <c r="A22" s="13">
         <v>46263</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="14">
         <v>480</v>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="14">
         <v>15</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="14">
         <v>40</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="14">
         <v>50</v>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="14">
         <v>0</v>
       </c>
-      <c r="G22" s="15">
+      <c r="G22" s="14">
         <v>0</v>
       </c>
-      <c r="H22" s="15">
+      <c r="H22" s="14">
         <v>100</v>
       </c>
-      <c r="I22" s="16">
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
         <v>685</v>
       </c>
-      <c r="J22" s="16">
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
         <v>755</v>
       </c>
-      <c r="K22" s="17" t="s">
+      <c r="K22" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L22" s="17" t="s">
+      <c r="L22" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M22" s="17" t="s">
+      <c r="M22" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N22" s="17" t="s">
+      <c r="N22" s="16" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="14">
+      <c r="A23" s="13">
         <v>46264</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="14">
         <v>360</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="14">
         <v>10</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="14">
         <v>30</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="14">
         <v>40</v>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="14">
         <v>0</v>
       </c>
-      <c r="G23" s="15">
+      <c r="G23" s="14">
         <v>0</v>
       </c>
-      <c r="H23" s="15">
+      <c r="H23" s="14">
         <v>120</v>
       </c>
-      <c r="I23" s="16">
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
         <v>560</v>
       </c>
-      <c r="J23" s="16">
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
         <v>880</v>
       </c>
-      <c r="K23" s="17" t="s">
+      <c r="K23" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L23" s="17" t="s">
+      <c r="L23" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M23" s="17" t="s">
+      <c r="M23" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N23" s="17" t="s">
+      <c r="N23" s="16" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="14">
+      <c r="A24" s="13">
         <v>46265</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="14">
         <v>420</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="14">
         <v>20</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="14">
         <v>25</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="14">
         <v>55</v>
       </c>
-      <c r="F24" s="15">
+      <c r="F24" s="14">
         <v>200</v>
       </c>
-      <c r="G24" s="15">
+      <c r="G24" s="14">
         <v>4</v>
       </c>
-      <c r="H24" s="15">
+      <c r="H24" s="14">
         <v>45</v>
       </c>
-      <c r="I24" s="16">
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
         <v>765</v>
       </c>
-      <c r="J24" s="16">
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
         <v>675</v>
       </c>
-      <c r="K24" s="17" t="s">
+      <c r="K24" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L24" s="17" t="s">
+      <c r="L24" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M24" s="17" t="s">
+      <c r="M24" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N24" s="17" t="s">
+      <c r="N24" s="16" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="14">
+      <c r="A25" s="13">
         <v>46266</v>
       </c>
-      <c r="B25" s="15">
+      <c r="B25" s="14">
         <v>375</v>
       </c>
-      <c r="C25" s="15">
+      <c r="C25" s="14">
         <v>10</v>
       </c>
-      <c r="D25" s="15">
+      <c r="D25" s="14">
         <v>20</v>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="14">
         <v>120</v>
       </c>
-      <c r="F25" s="15">
+      <c r="F25" s="14">
         <v>200</v>
       </c>
-      <c r="G25" s="15">
+      <c r="G25" s="14">
         <v>4</v>
       </c>
-      <c r="H25" s="15">
+      <c r="H25" s="14">
         <v>200</v>
       </c>
-      <c r="I25" s="16">
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
         <v>925</v>
       </c>
-      <c r="J25" s="16">
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
         <v>515</v>
       </c>
-      <c r="K25" s="17" t="s">
+      <c r="K25" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L25" s="17" t="s">
+      <c r="L25" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M25" s="17" t="s">
+      <c r="M25" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N25" s="17" t="s">
+      <c r="N25" s="16" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="14">
+      <c r="A26" s="13">
         <v>46267</v>
       </c>
-      <c r="B26" s="15">
+      <c r="B26" s="14">
         <v>390</v>
       </c>
-      <c r="C26" s="15">
+      <c r="C26" s="14">
         <v>15</v>
       </c>
-      <c r="D26" s="15">
+      <c r="D26" s="14">
         <v>40</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="14">
         <v>100</v>
       </c>
-      <c r="F26" s="15">
+      <c r="F26" s="14">
         <v>250</v>
       </c>
-      <c r="G26" s="15">
+      <c r="G26" s="14">
         <v>5</v>
       </c>
-      <c r="H26" s="15">
+      <c r="H26" s="14">
         <v>40</v>
       </c>
-      <c r="I26" s="16">
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
         <v>835</v>
       </c>
-      <c r="J26" s="16">
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
         <v>605</v>
       </c>
-      <c r="K26" s="17" t="s">
+      <c r="K26" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L26" s="17" t="s">
+      <c r="L26" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M26" s="17" t="s">
+      <c r="M26" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N26" s="17" t="s">
+      <c r="N26" s="16" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="14">
+      <c r="A27" s="13">
         <v>46268</v>
       </c>
-      <c r="B27" s="15">
+      <c r="B27" s="14">
         <v>420</v>
       </c>
-      <c r="C27" s="15">
+      <c r="C27" s="14">
         <v>25</v>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="14">
         <v>35</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="14">
         <v>45</v>
       </c>
-      <c r="F27" s="15">
+      <c r="F27" s="14">
         <v>360</v>
       </c>
-      <c r="G27" s="15">
+      <c r="G27" s="14">
         <v>6</v>
       </c>
-      <c r="H27" s="15">
+      <c r="H27" s="14">
         <v>90</v>
       </c>
-      <c r="I27" s="16">
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
         <v>975</v>
       </c>
-      <c r="J27" s="16">
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
         <v>465</v>
       </c>
-      <c r="K27" s="17" t="s">
+      <c r="K27" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="L27" s="17" t="s">
+      <c r="L27" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="M27" s="17" t="s">
+      <c r="M27" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N27" s="17" t="s">
+      <c r="N27" s="16" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="14">
+      <c r="A28" s="13">
         <v>46269</v>
       </c>
-      <c r="B28" s="15">
+      <c r="B28" s="14">
         <v>330</v>
       </c>
-      <c r="C28" s="15">
+      <c r="C28" s="14">
         <v>30</v>
       </c>
-      <c r="D28" s="15">
+      <c r="D28" s="14">
         <v>50</v>
       </c>
-      <c r="E28" s="15">
+      <c r="E28" s="14">
         <v>35</v>
       </c>
-      <c r="F28" s="15">
+      <c r="F28" s="14">
         <v>350</v>
       </c>
-      <c r="G28" s="15">
+      <c r="G28" s="14">
         <v>7</v>
       </c>
-      <c r="H28" s="15">
+      <c r="H28" s="14">
         <v>79</v>
       </c>
-      <c r="I28" s="16">
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
         <v>874</v>
       </c>
-      <c r="J28" s="16">
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
         <v>566</v>
       </c>
-      <c r="K28" s="17" t="s">
+      <c r="K28" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L28" s="17" t="s">
+      <c r="L28" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="M28" s="17" t="s">
+      <c r="M28" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N28" s="17" t="s">
+      <c r="N28" s="16" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="14">
+      <c r="A29" s="13">
         <v>46270</v>
       </c>
-      <c r="B29" s="15">
+      <c r="B29" s="14">
         <v>480</v>
       </c>
-      <c r="C29" s="15">
+      <c r="C29" s="14">
         <v>0</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="14">
         <v>10</v>
       </c>
-      <c r="E29" s="15">
+      <c r="E29" s="14">
         <v>20</v>
       </c>
-      <c r="F29" s="15">
+      <c r="F29" s="14">
         <v>0</v>
       </c>
-      <c r="G29" s="15">
+      <c r="G29" s="14">
         <v>0</v>
       </c>
-      <c r="H29" s="15">
+      <c r="H29" s="14">
         <v>180</v>
       </c>
-      <c r="I29" s="16">
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
         <v>690</v>
       </c>
-      <c r="J29" s="16">
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
         <v>750</v>
       </c>
-      <c r="K29" s="17" t="s">
+      <c r="K29" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L29" s="17" t="s">
+      <c r="L29" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M29" s="17" t="s">
+      <c r="M29" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N29" s="17" t="s">
+      <c r="N29" s="16" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A30" s="14">
+      <c r="A30" s="13">
         <v>46271</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="14">
         <v>450</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="14">
         <v>0</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="14">
         <v>20</v>
       </c>
-      <c r="E30" s="15">
+      <c r="E30" s="14">
         <v>30</v>
       </c>
-      <c r="F30" s="15">
+      <c r="F30" s="14">
         <v>0</v>
       </c>
-      <c r="G30" s="15">
+      <c r="G30" s="14">
         <v>0</v>
       </c>
-      <c r="H30" s="15">
+      <c r="H30" s="14">
         <v>120</v>
       </c>
-      <c r="I30" s="16">
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
         <v>620</v>
       </c>
-      <c r="J30" s="16">
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
         <v>820</v>
       </c>
-      <c r="K30" s="17" t="s">
+      <c r="K30" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L30" s="17" t="s">
+      <c r="L30" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="M30" s="17" t="s">
+      <c r="M30" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="N30" s="17" t="s">
+      <c r="N30" s="16" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A31" s="14">
+      <c r="A31" s="13">
         <v>46272</v>
       </c>
-      <c r="B31" s="15">
+      <c r="B31" s="14">
         <v>330</v>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="14">
         <v>20</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="14">
         <v>40</v>
       </c>
-      <c r="E31" s="15">
+      <c r="E31" s="14">
         <v>40</v>
       </c>
-      <c r="F31" s="15">
+      <c r="F31" s="14">
         <v>250</v>
       </c>
-      <c r="G31" s="15">
+      <c r="G31" s="14">
         <v>5</v>
       </c>
-      <c r="H31" s="15">
+      <c r="H31" s="14">
         <v>80</v>
       </c>
-      <c r="I31" s="16">
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
         <v>760</v>
       </c>
-      <c r="J31" s="16">
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
         <v>680</v>
       </c>
-      <c r="K31" s="17" t="s">
+      <c r="K31" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="L31" s="17" t="s">
+      <c r="L31" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M31" s="17" t="s">
+      <c r="M31" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N31" s="17" t="s">
+      <c r="N31" s="16" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="14">
+      <c r="A32" s="13">
         <v>46273</v>
       </c>
-      <c r="B32" s="15">
+      <c r="B32" s="14">
         <v>360</v>
       </c>
-      <c r="C32" s="15">
+      <c r="C32" s="14">
         <v>30</v>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="14">
         <v>50</v>
       </c>
-      <c r="E32" s="15">
+      <c r="E32" s="14">
         <v>50</v>
       </c>
-      <c r="F32" s="15">
+      <c r="F32" s="14">
         <v>250</v>
       </c>
-      <c r="G32" s="15">
+      <c r="G32" s="14">
         <v>5</v>
       </c>
-      <c r="H32" s="15">
+      <c r="H32" s="14">
         <v>240</v>
       </c>
-      <c r="I32" s="16">
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
         <v>980</v>
       </c>
-      <c r="J32" s="16">
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
         <v>460</v>
       </c>
-      <c r="K32" s="17" t="s">
+      <c r="K32" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L32" s="17" t="s">
+      <c r="L32" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="M32" s="17" t="s">
+      <c r="M32" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N32" s="17" t="s">
+      <c r="N32" s="16" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A33" s="14">
+      <c r="A33" s="13">
         <v>46274</v>
       </c>
-      <c r="B33" s="15">
+      <c r="B33" s="14">
         <v>350</v>
       </c>
-      <c r="C33" s="15">
+      <c r="C33" s="14">
         <v>20</v>
       </c>
-      <c r="D33" s="15">
+      <c r="D33" s="14">
         <v>40</v>
       </c>
-      <c r="E33" s="15">
+      <c r="E33" s="14">
         <v>60</v>
       </c>
-      <c r="F33" s="15">
+      <c r="F33" s="14">
         <v>250</v>
       </c>
-      <c r="G33" s="15">
+      <c r="G33" s="14">
         <v>5</v>
       </c>
-      <c r="H33" s="15">
+      <c r="H33" s="14">
         <v>60</v>
       </c>
-      <c r="I33" s="16">
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
         <v>780</v>
       </c>
-      <c r="J33" s="16">
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
         <v>660</v>
       </c>
-      <c r="K33" s="17" t="s">
+      <c r="K33" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L33" s="17" t="s">
+      <c r="L33" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M33" s="17" t="s">
+      <c r="M33" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="N33" s="17" t="s">
+      <c r="N33" s="16" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A34" s="14">
+      <c r="A34" s="13">
         <v>46275</v>
       </c>
-      <c r="B34" s="15">
+      <c r="B34" s="14">
         <v>380</v>
       </c>
-      <c r="C34" s="15">
+      <c r="C34" s="14">
         <v>30</v>
       </c>
-      <c r="D34" s="15">
+      <c r="D34" s="14">
         <v>80</v>
       </c>
-      <c r="E34" s="15">
+      <c r="E34" s="14">
         <v>10</v>
       </c>
-      <c r="F34" s="15">
+      <c r="F34" s="14">
         <v>100</v>
       </c>
-      <c r="G34" s="15">
+      <c r="G34" s="14">
         <v>2</v>
       </c>
-      <c r="H34" s="15">
+      <c r="H34" s="14">
         <v>15</v>
       </c>
-      <c r="I34" s="16">
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
         <v>615</v>
       </c>
-      <c r="J34" s="16">
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
         <v>825</v>
       </c>
-      <c r="K34" s="17" t="s">
+      <c r="K34" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L34" s="17" t="s">
+      <c r="L34" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M34" s="17" t="s">
+      <c r="M34" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N34" s="17" t="s">
+      <c r="N34" s="16" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="14">
+      <c r="A35" s="13">
         <v>46276</v>
       </c>
-      <c r="B35" s="15">
+      <c r="B35" s="14">
         <v>410</v>
       </c>
-      <c r="C35" s="15">
+      <c r="C35" s="14">
         <v>20</v>
       </c>
-      <c r="D35" s="15">
+      <c r="D35" s="14">
         <v>40</v>
       </c>
-      <c r="E35" s="15">
+      <c r="E35" s="14">
         <v>50</v>
       </c>
-      <c r="F35" s="15">
+      <c r="F35" s="14">
         <v>300</v>
       </c>
-      <c r="G35" s="15">
+      <c r="G35" s="14">
         <v>6</v>
       </c>
-      <c r="H35" s="15">
+      <c r="H35" s="14">
         <v>60</v>
       </c>
-      <c r="I35" s="16">
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
         <v>880</v>
       </c>
-      <c r="J35" s="16">
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
         <v>560</v>
       </c>
-      <c r="K35" s="17" t="s">
+      <c r="K35" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L35" s="17" t="s">
+      <c r="L35" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M35" s="17" t="s">
+      <c r="M35" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N35" s="17" t="s">
+      <c r="N35" s="16" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="14">
+      <c r="A36" s="13">
         <v>46277</v>
       </c>
-      <c r="B36" s="15">
+      <c r="B36" s="14">
         <v>450</v>
       </c>
-      <c r="C36" s="15">
+      <c r="C36" s="14">
         <v>10</v>
       </c>
-      <c r="D36" s="15">
+      <c r="D36" s="14">
         <v>15</v>
       </c>
-      <c r="E36" s="15">
+      <c r="E36" s="14">
         <v>30</v>
       </c>
-      <c r="F36" s="15">
+      <c r="F36" s="14">
         <v>0</v>
       </c>
-      <c r="G36" s="15">
+      <c r="G36" s="14">
         <v>0</v>
       </c>
-      <c r="H36" s="15">
+      <c r="H36" s="14">
         <v>240</v>
       </c>
-      <c r="I36" s="16">
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
         <v>745</v>
       </c>
-      <c r="J36" s="16">
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
         <v>695</v>
       </c>
-      <c r="K36" s="17" t="s">
+      <c r="K36" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L36" s="17" t="s">
+      <c r="L36" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M36" s="17" t="s">
+      <c r="M36" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="N36" s="17" t="s">
+      <c r="N36" s="16" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="14">
+      <c r="A37" s="13">
         <v>46278</v>
       </c>
-      <c r="B37" s="15">
+      <c r="B37" s="14">
         <v>300</v>
       </c>
-      <c r="C37" s="15">
+      <c r="C37" s="14">
         <v>0</v>
       </c>
-      <c r="D37" s="15">
+      <c r="D37" s="14">
         <v>20</v>
       </c>
-      <c r="E37" s="15">
+      <c r="E37" s="14">
         <v>50</v>
       </c>
-      <c r="F37" s="15">
+      <c r="F37" s="14">
         <v>0</v>
       </c>
-      <c r="G37" s="15">
+      <c r="G37" s="14">
         <v>0</v>
       </c>
-      <c r="H37" s="15">
+      <c r="H37" s="14">
         <v>300</v>
       </c>
-      <c r="I37" s="16">
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
         <v>670</v>
       </c>
-      <c r="J37" s="16">
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
         <v>770</v>
       </c>
-      <c r="K37" s="17" t="s">
+      <c r="K37" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L37" s="17" t="s">
+      <c r="L37" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="M37" s="17" t="s">
+      <c r="M37" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N37" s="17" t="s">
+      <c r="N37" s="16" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A38" s="14">
+      <c r="A38" s="13">
         <v>46279</v>
       </c>
-      <c r="B38" s="15">
+      <c r="B38" s="14">
         <v>420</v>
       </c>
-      <c r="C38" s="15">
+      <c r="C38" s="14">
         <v>15</v>
       </c>
-      <c r="D38" s="15">
+      <c r="D38" s="14">
         <v>40</v>
       </c>
-      <c r="E38" s="15">
+      <c r="E38" s="14">
         <v>60</v>
       </c>
-      <c r="F38" s="15">
+      <c r="F38" s="14">
         <v>200</v>
       </c>
-      <c r="G38" s="15">
+      <c r="G38" s="14">
         <v>4</v>
       </c>
-      <c r="H38" s="15">
+      <c r="H38" s="14">
         <v>200</v>
       </c>
-      <c r="I38" s="16">
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
         <v>935</v>
       </c>
-      <c r="J38" s="16">
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
         <v>505</v>
       </c>
-      <c r="K38" s="17" t="s">
+      <c r="K38" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="L38" s="17" t="s">
+      <c r="L38" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="M38" s="17" t="s">
+      <c r="M38" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N38" s="17" t="s">
+      <c r="N38" s="16" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A39" s="14">
+      <c r="A39" s="13">
         <v>46280</v>
       </c>
-      <c r="B39" s="15">
+      <c r="B39" s="14">
         <v>330</v>
       </c>
-      <c r="C39" s="15">
+      <c r="C39" s="14">
         <v>10</v>
       </c>
-      <c r="D39" s="15">
+      <c r="D39" s="14">
         <v>20</v>
       </c>
-      <c r="E39" s="15">
+      <c r="E39" s="14">
         <v>40</v>
       </c>
-      <c r="F39" s="15">
+      <c r="F39" s="14">
         <v>250</v>
       </c>
-      <c r="G39" s="15">
+      <c r="G39" s="14">
         <v>5</v>
       </c>
-      <c r="H39" s="15">
+      <c r="H39" s="14">
         <v>150</v>
       </c>
-      <c r="I39" s="16">
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
         <v>800</v>
       </c>
-      <c r="J39" s="16">
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
         <v>640</v>
       </c>
-      <c r="K39" s="17" t="s">
+      <c r="K39" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="L39" s="17" t="s">
+      <c r="L39" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M39" s="17" t="s">
+      <c r="M39" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N39" s="17" t="s">
+      <c r="N39" s="16" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A40" s="14">
+      <c r="A40" s="13">
         <v>46281</v>
       </c>
-      <c r="B40" s="15">
+      <c r="B40" s="14">
         <v>510</v>
       </c>
-      <c r="C40" s="15">
+      <c r="C40" s="14">
         <v>0</v>
       </c>
-      <c r="D40" s="15">
+      <c r="D40" s="14">
         <v>60</v>
       </c>
-      <c r="E40" s="15">
+      <c r="E40" s="14">
         <v>30</v>
       </c>
-      <c r="F40" s="15">
+      <c r="F40" s="14">
         <v>250</v>
       </c>
-      <c r="G40" s="15">
+      <c r="G40" s="14">
         <v>5</v>
       </c>
-      <c r="H40" s="15">
+      <c r="H40" s="14">
         <v>90</v>
       </c>
-      <c r="I40" s="16">
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
         <v>940</v>
       </c>
-      <c r="J40" s="16">
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="K40" s="17" t="s">
+      <c r="K40" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L40" s="17" t="s">
+      <c r="L40" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M40" s="17" t="s">
+      <c r="M40" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N40" s="17" t="s">
+      <c r="N40" s="16" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="14">
+      <c r="A41" s="13">
         <v>46282</v>
       </c>
-      <c r="B41" s="15">
+      <c r="B41" s="14">
         <v>290</v>
       </c>
-      <c r="C41" s="15">
+      <c r="C41" s="14">
         <v>10</v>
       </c>
-      <c r="D41" s="15">
+      <c r="D41" s="14">
         <v>45</v>
       </c>
-      <c r="E41" s="15">
+      <c r="E41" s="14">
         <v>30</v>
       </c>
-      <c r="F41" s="15">
+      <c r="F41" s="14">
         <v>300</v>
       </c>
-      <c r="G41" s="15">
+      <c r="G41" s="14">
         <v>6</v>
       </c>
-      <c r="H41" s="15">
+      <c r="H41" s="14">
         <v>60</v>
       </c>
-      <c r="I41" s="16">
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
         <v>735</v>
       </c>
-      <c r="J41" s="16">
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
         <v>705</v>
       </c>
-      <c r="K41" s="17" t="s">
+      <c r="K41" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L41" s="17" t="s">
+      <c r="L41" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M41" s="17" t="s">
+      <c r="M41" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N41" s="17" t="s">
+      <c r="N41" s="16" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="14">
+      <c r="A42" s="13">
         <v>46283</v>
       </c>
-      <c r="B42" s="15">
+      <c r="B42" s="14">
         <v>350</v>
       </c>
-      <c r="C42" s="15">
+      <c r="C42" s="14">
         <v>15</v>
       </c>
-      <c r="D42" s="15">
+      <c r="D42" s="14">
         <v>40</v>
       </c>
-      <c r="E42" s="15">
+      <c r="E42" s="14">
         <v>45</v>
       </c>
-      <c r="F42" s="15">
+      <c r="F42" s="14">
         <v>350</v>
       </c>
-      <c r="G42" s="15">
+      <c r="G42" s="14">
         <v>7</v>
       </c>
-      <c r="H42" s="15">
+      <c r="H42" s="14">
         <v>90</v>
       </c>
-      <c r="I42" s="16">
+      <c r="I42" s="15">
         <f t="shared" si="0"/>
         <v>890</v>
       </c>
-      <c r="J42" s="16">
+      <c r="J42" s="15">
         <f t="shared" si="1"/>
         <v>550</v>
       </c>
-      <c r="K42" s="17" t="s">
+      <c r="K42" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L42" s="17" t="s">
+      <c r="L42" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M42" s="17" t="s">
+      <c r="M42" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N42" s="17" t="s">
+      <c r="N42" s="16" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="72" x14ac:dyDescent="0.3">
-      <c r="A43" s="14">
+      <c r="A43" s="13">
         <v>46284</v>
       </c>
-      <c r="B43" s="15">
+      <c r="B43" s="14">
         <v>240</v>
       </c>
-      <c r="C43" s="15">
+      <c r="C43" s="14">
         <v>10</v>
       </c>
-      <c r="D43" s="15">
+      <c r="D43" s="14">
         <v>20</v>
       </c>
-      <c r="E43" s="15">
+      <c r="E43" s="14">
         <v>10</v>
       </c>
-      <c r="F43" s="15">
+      <c r="F43" s="14">
         <v>60</v>
       </c>
-      <c r="G43" s="15">
+      <c r="G43" s="14">
         <v>1</v>
       </c>
-      <c r="H43" s="15">
+      <c r="H43" s="14">
         <v>360</v>
       </c>
-      <c r="I43" s="16">
+      <c r="I43" s="15">
         <f t="shared" si="0"/>
         <v>700</v>
       </c>
-      <c r="J43" s="16">
+      <c r="J43" s="15">
         <f t="shared" si="1"/>
         <v>740</v>
       </c>
-      <c r="K43" s="17" t="s">
+      <c r="K43" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="L43" s="17" t="s">
+      <c r="L43" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="M43" s="17" t="s">
+      <c r="M43" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N43" s="17" t="s">
+      <c r="N43" s="16" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A44" s="14">
+      <c r="A44" s="13">
         <v>46285</v>
       </c>
-      <c r="B44" s="15">
+      <c r="B44" s="14">
         <v>410</v>
       </c>
-      <c r="C44" s="15">
+      <c r="C44" s="14">
         <v>0</v>
       </c>
-      <c r="D44" s="15">
+      <c r="D44" s="14">
         <v>70</v>
       </c>
-      <c r="E44" s="15">
+      <c r="E44" s="14">
         <v>50</v>
       </c>
-      <c r="F44" s="15">
+      <c r="F44" s="14">
         <v>0</v>
       </c>
-      <c r="G44" s="15">
+      <c r="G44" s="14">
         <v>0</v>
       </c>
-      <c r="H44" s="15">
+      <c r="H44" s="14">
         <v>410</v>
       </c>
-      <c r="I44" s="16">
+      <c r="I44" s="15">
         <f t="shared" si="0"/>
         <v>940</v>
       </c>
-      <c r="J44" s="16">
+      <c r="J44" s="15">
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="K44" s="17" t="s">
+      <c r="K44" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="L44" s="17" t="s">
+      <c r="L44" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="M44" s="17" t="s">
+      <c r="M44" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N44" s="17" t="s">
+      <c r="N44" s="16" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="14">
+      <c r="A45" s="13">
         <v>46286</v>
       </c>
-      <c r="B45" s="15">
+      <c r="B45" s="14">
         <v>350</v>
       </c>
-      <c r="C45" s="15">
+      <c r="C45" s="14">
         <v>30</v>
       </c>
-      <c r="D45" s="15">
+      <c r="D45" s="14">
         <v>40</v>
       </c>
-      <c r="E45" s="15">
+      <c r="E45" s="14">
         <v>60</v>
       </c>
-      <c r="F45" s="15">
+      <c r="F45" s="14">
         <v>200</v>
       </c>
-      <c r="G45" s="15">
+      <c r="G45" s="14">
         <v>4</v>
       </c>
-      <c r="H45" s="15">
+      <c r="H45" s="14">
         <v>150</v>
       </c>
-      <c r="I45" s="16">
+      <c r="I45" s="15">
         <f t="shared" si="0"/>
         <v>830</v>
       </c>
-      <c r="J45" s="16">
+      <c r="J45" s="15">
         <f t="shared" si="1"/>
         <v>610</v>
       </c>
-      <c r="K45" s="17" t="s">
+      <c r="K45" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="L45" s="17" t="s">
+      <c r="L45" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="M45" s="17" t="s">
+      <c r="M45" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="N45" s="17" t="s">
+      <c r="N45" s="16" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="8"/>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9"/>
-      <c r="G46" s="9"/>
-      <c r="H46" s="9"/>
-      <c r="I46" s="10" t="str">
+    <row r="46" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="8">
+        <v>46287</v>
+      </c>
+      <c r="B46" s="9">
+        <v>300</v>
+      </c>
+      <c r="C46" s="9">
+        <v>20</v>
+      </c>
+      <c r="D46" s="9">
+        <v>60</v>
+      </c>
+      <c r="E46" s="9">
+        <v>60</v>
+      </c>
+      <c r="F46" s="9">
+        <v>250</v>
+      </c>
+      <c r="G46" s="9">
+        <v>5</v>
+      </c>
+      <c r="H46" s="9">
+        <v>220</v>
+      </c>
+      <c r="I46" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="10" t="str">
+        <v>910</v>
+      </c>
+      <c r="J46" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="11"/>
-      <c r="L46" s="11"/>
-      <c r="M46" s="11"/>
-      <c r="N46" s="12"/>
+        <v>530</v>
+      </c>
+      <c r="K46" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L46" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="M46" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="N46" s="12" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="8"/>
@@ -10998,7 +10989,7 @@
     <mergeCell ref="F3:G3"/>
   </mergeCells>
   <conditionalFormatting sqref="J6:J406">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Updated Daily Excel Data.
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C47538D4-19DA-4207-ADD0-4501E0A4DDEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172332AC-DC4F-416F-BC19-BA5A64E9AC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="133">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -376,7 +376,64 @@
     <t>Working on DSA Concept Infix to Postfix Conversion.</t>
   </si>
   <si>
-    <t>Working on DSA Conecpt Postifix Evalucation.</t>
+    <t>Today I did well in my networking Exam.</t>
+  </si>
+  <si>
+    <t>I need to focus more on C++ Advace concept. Could have done better in Exam.</t>
+  </si>
+  <si>
+    <t>DBMS Exam was very easy. Need to work hard for final of DBMS.</t>
+  </si>
+  <si>
+    <t>Tomorrow is Analytical Skill exam. It's very tough.</t>
+  </si>
+  <si>
+    <t>I didn't do well on my exam. I should have studied more.</t>
+  </si>
+  <si>
+    <t>I did okay I today's english exam. Will focus on grammer.</t>
+  </si>
+  <si>
+    <t>Today I relaxed and did nothing important.</t>
+  </si>
+  <si>
+    <t>I only got one day break after exam.</t>
+  </si>
+  <si>
+    <t>Enjoyed the Dussehra Mela with my friend.</t>
+  </si>
+  <si>
+    <t>C++ will have Project as CA instread of Exams.</t>
+  </si>
+  <si>
+    <t>Today was our first online class and it went well.</t>
+  </si>
+  <si>
+    <t>Preparing for my upcoming exams.</t>
+  </si>
+  <si>
+    <t>Need to do better in Networking Practicals.</t>
+  </si>
+  <si>
+    <t>Need to prepare DBMS Theory</t>
+  </si>
+  <si>
+    <t>Tried to python oops programming.</t>
+  </si>
+  <si>
+    <t>Today's online class was optional still attended it.</t>
+  </si>
+  <si>
+    <t>From Tomorrow onwards online classes will be held.</t>
+  </si>
+  <si>
+    <t>Need to prepare for my upcoming exams.</t>
+  </si>
+  <si>
+    <t>Working on DSA Conecpt Postifix Evaluation.</t>
+  </si>
+  <si>
+    <t>Concept of postfix and infix evaluation.</t>
   </si>
 </sst>
 </file>
@@ -3495,450 +3552,928 @@
         <v>55</v>
       </c>
       <c r="N55" s="16" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A56" s="13">
+        <v>46297</v>
+      </c>
+      <c r="B56" s="14">
+        <v>480</v>
+      </c>
+      <c r="C56" s="14">
+        <v>15</v>
+      </c>
+      <c r="D56" s="14">
+        <v>60</v>
+      </c>
+      <c r="E56" s="14">
+        <v>60</v>
+      </c>
+      <c r="F56" s="14">
+        <v>0</v>
+      </c>
+      <c r="G56" s="14">
+        <v>0</v>
+      </c>
+      <c r="H56" s="14">
+        <v>190</v>
+      </c>
+      <c r="I56" s="15">
+        <f t="shared" si="2"/>
+        <v>805</v>
+      </c>
+      <c r="J56" s="15">
+        <f t="shared" si="3"/>
+        <v>635</v>
+      </c>
+      <c r="K56" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L56" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M56" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N56" s="16" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A57" s="13">
+        <v>46298</v>
+      </c>
+      <c r="B57" s="14">
+        <v>470</v>
+      </c>
+      <c r="C57" s="14">
+        <v>20</v>
+      </c>
+      <c r="D57" s="14">
+        <v>50</v>
+      </c>
+      <c r="E57" s="14">
+        <v>80</v>
+      </c>
+      <c r="F57" s="14">
+        <v>0</v>
+      </c>
+      <c r="G57" s="14">
+        <v>0</v>
+      </c>
+      <c r="H57" s="14">
+        <v>260</v>
+      </c>
+      <c r="I57" s="15">
+        <f t="shared" si="2"/>
+        <v>880</v>
+      </c>
+      <c r="J57" s="15">
+        <f t="shared" si="3"/>
+        <v>560</v>
+      </c>
+      <c r="K57" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L57" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M57" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N57" s="16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A58" s="13">
+        <v>46299</v>
+      </c>
+      <c r="B58" s="14">
+        <v>490</v>
+      </c>
+      <c r="C58" s="14">
+        <v>25</v>
+      </c>
+      <c r="D58" s="14">
+        <v>40</v>
+      </c>
+      <c r="E58" s="14">
+        <v>40</v>
+      </c>
+      <c r="F58" s="14">
+        <v>0</v>
+      </c>
+      <c r="G58" s="14">
+        <v>0</v>
+      </c>
+      <c r="H58" s="14">
+        <v>240</v>
+      </c>
+      <c r="I58" s="15">
+        <f t="shared" si="2"/>
+        <v>835</v>
+      </c>
+      <c r="J58" s="15">
+        <f t="shared" si="3"/>
+        <v>605</v>
+      </c>
+      <c r="K58" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L58" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M58" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N58" s="16" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A59" s="13">
+        <v>46300</v>
+      </c>
+      <c r="B59" s="14">
+        <v>420</v>
+      </c>
+      <c r="C59" s="14">
+        <v>20</v>
+      </c>
+      <c r="D59" s="14">
+        <v>30</v>
+      </c>
+      <c r="E59" s="14">
+        <v>30</v>
+      </c>
+      <c r="F59" s="14">
+        <v>200</v>
+      </c>
+      <c r="G59" s="14">
+        <v>4</v>
+      </c>
+      <c r="H59" s="14">
+        <v>180</v>
+      </c>
+      <c r="I59" s="15">
+        <f t="shared" si="2"/>
+        <v>880</v>
+      </c>
+      <c r="J59" s="15">
+        <f t="shared" si="3"/>
+        <v>560</v>
+      </c>
+      <c r="K59" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L59" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M59" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N59" s="16" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A60" s="13">
+        <v>46301</v>
+      </c>
+      <c r="B60" s="14">
+        <v>410</v>
+      </c>
+      <c r="C60" s="14">
+        <v>25</v>
+      </c>
+      <c r="D60" s="14">
+        <v>40</v>
+      </c>
+      <c r="E60" s="14">
+        <v>60</v>
+      </c>
+      <c r="F60" s="14">
+        <v>250</v>
+      </c>
+      <c r="G60" s="14">
+        <v>5</v>
+      </c>
+      <c r="H60" s="14">
+        <v>70</v>
+      </c>
+      <c r="I60" s="15">
+        <f t="shared" si="2"/>
+        <v>855</v>
+      </c>
+      <c r="J60" s="15">
+        <f t="shared" si="3"/>
+        <v>585</v>
+      </c>
+      <c r="K60" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L60" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M60" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N60" s="16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A61" s="13">
+        <v>46302</v>
+      </c>
+      <c r="B61" s="14">
+        <v>390</v>
+      </c>
+      <c r="C61" s="14">
+        <v>20</v>
+      </c>
+      <c r="D61" s="14">
+        <v>50</v>
+      </c>
+      <c r="E61" s="14">
+        <v>40</v>
+      </c>
+      <c r="F61" s="14">
+        <v>250</v>
+      </c>
+      <c r="G61" s="14">
+        <v>5</v>
+      </c>
+      <c r="H61" s="14">
+        <v>190</v>
+      </c>
+      <c r="I61" s="15">
+        <f t="shared" si="2"/>
+        <v>940</v>
+      </c>
+      <c r="J61" s="15">
+        <f t="shared" si="3"/>
+        <v>500</v>
+      </c>
+      <c r="K61" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L61" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M61" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N61" s="16" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A62" s="13">
+        <v>46303</v>
+      </c>
+      <c r="B62" s="14">
+        <v>370</v>
+      </c>
+      <c r="C62" s="14">
+        <v>20</v>
+      </c>
+      <c r="D62" s="14">
+        <v>60</v>
+      </c>
+      <c r="E62" s="14">
+        <v>60</v>
+      </c>
+      <c r="F62" s="14">
+        <v>300</v>
+      </c>
+      <c r="G62" s="14">
+        <v>6</v>
+      </c>
+      <c r="H62" s="14">
+        <v>70</v>
+      </c>
+      <c r="I62" s="15">
+        <f t="shared" si="2"/>
+        <v>880</v>
+      </c>
+      <c r="J62" s="15">
+        <f t="shared" si="3"/>
+        <v>560</v>
+      </c>
+      <c r="K62" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L62" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M62" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N62" s="16" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A63" s="13">
+        <v>46304</v>
+      </c>
+      <c r="B63" s="14">
+        <v>380</v>
+      </c>
+      <c r="C63" s="14">
+        <v>25</v>
+      </c>
+      <c r="D63" s="14">
+        <v>50</v>
+      </c>
+      <c r="E63" s="14">
+        <v>35</v>
+      </c>
+      <c r="F63" s="14">
+        <v>350</v>
+      </c>
+      <c r="G63" s="14">
+        <v>7</v>
+      </c>
+      <c r="H63" s="14">
+        <v>260</v>
+      </c>
+      <c r="I63" s="15">
+        <f t="shared" si="2"/>
+        <v>1100</v>
+      </c>
+      <c r="J63" s="15">
+        <f t="shared" si="3"/>
+        <v>340</v>
+      </c>
+      <c r="K63" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L63" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M63" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N63" s="16" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A64" s="13">
+        <v>46305</v>
+      </c>
+      <c r="B64" s="14">
+        <v>450</v>
+      </c>
+      <c r="C64" s="14">
+        <v>15</v>
+      </c>
+      <c r="D64" s="14">
+        <v>190</v>
+      </c>
+      <c r="E64" s="14">
+        <v>20</v>
+      </c>
+      <c r="F64" s="14">
+        <v>0</v>
+      </c>
+      <c r="G64" s="14">
+        <v>0</v>
+      </c>
+      <c r="H64" s="14">
+        <v>240</v>
+      </c>
+      <c r="I64" s="15">
+        <f t="shared" si="2"/>
+        <v>915</v>
+      </c>
+      <c r="J64" s="15">
+        <f t="shared" si="3"/>
+        <v>525</v>
+      </c>
+      <c r="K64" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L64" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M64" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N64" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A65" s="13">
+        <v>46306</v>
+      </c>
+      <c r="B65" s="14">
+        <v>350</v>
+      </c>
+      <c r="C65" s="14">
+        <v>20</v>
+      </c>
+      <c r="D65" s="14">
+        <v>320</v>
+      </c>
+      <c r="E65" s="14">
+        <v>30</v>
+      </c>
+      <c r="F65" s="14">
+        <v>0</v>
+      </c>
+      <c r="G65" s="14">
+        <v>0</v>
+      </c>
+      <c r="H65" s="14">
+        <v>190</v>
+      </c>
+      <c r="I65" s="15">
+        <f t="shared" si="2"/>
+        <v>910</v>
+      </c>
+      <c r="J65" s="15">
+        <f t="shared" si="3"/>
+        <v>530</v>
+      </c>
+      <c r="K65" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L65" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M65" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N65" s="16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A66" s="13">
+        <v>46307</v>
+      </c>
+      <c r="B66" s="14">
+        <v>390</v>
+      </c>
+      <c r="C66" s="14">
+        <v>10</v>
+      </c>
+      <c r="D66" s="14">
+        <v>240</v>
+      </c>
+      <c r="E66" s="14">
+        <v>20</v>
+      </c>
+      <c r="F66" s="14">
+        <v>0</v>
+      </c>
+      <c r="G66" s="14">
+        <v>0</v>
+      </c>
+      <c r="H66" s="14">
+        <v>35</v>
+      </c>
+      <c r="I66" s="15">
+        <f t="shared" si="2"/>
+        <v>695</v>
+      </c>
+      <c r="J66" s="15">
+        <f t="shared" si="3"/>
+        <v>745</v>
+      </c>
+      <c r="K66" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L66" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M66" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N66" s="16" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="8">
-        <v>46297</v>
-      </c>
-      <c r="B56" s="9"/>
-      <c r="C56" s="9"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="9"/>
-      <c r="F56" s="9"/>
-      <c r="G56" s="9"/>
-      <c r="H56" s="9"/>
-      <c r="I56" s="10" t="str">
+    <row r="67" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A67" s="13">
+        <v>46308</v>
+      </c>
+      <c r="B67" s="14">
+        <v>410</v>
+      </c>
+      <c r="C67" s="14">
+        <v>15</v>
+      </c>
+      <c r="D67" s="14">
+        <v>270</v>
+      </c>
+      <c r="E67" s="14">
+        <v>40</v>
+      </c>
+      <c r="F67" s="14">
+        <v>0</v>
+      </c>
+      <c r="G67" s="14">
+        <v>0</v>
+      </c>
+      <c r="H67" s="14">
+        <v>40</v>
+      </c>
+      <c r="I67" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J56" s="10" t="str">
+        <v>775</v>
+      </c>
+      <c r="J67" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K56" s="11"/>
-      <c r="L56" s="11"/>
-      <c r="M56" s="11"/>
-      <c r="N56" s="12"/>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="8"/>
-      <c r="B57" s="9"/>
-      <c r="C57" s="9"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="9"/>
-      <c r="G57" s="9"/>
-      <c r="H57" s="9"/>
-      <c r="I57" s="10" t="str">
+        <v>665</v>
+      </c>
+      <c r="K67" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L67" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M67" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N67" s="16" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A68" s="13">
+        <v>46309</v>
+      </c>
+      <c r="B68" s="14">
+        <v>390</v>
+      </c>
+      <c r="C68" s="14">
+        <v>20</v>
+      </c>
+      <c r="D68" s="14">
+        <v>220</v>
+      </c>
+      <c r="E68" s="14">
+        <v>45</v>
+      </c>
+      <c r="F68" s="14">
+        <v>0</v>
+      </c>
+      <c r="G68" s="14">
+        <v>0</v>
+      </c>
+      <c r="H68" s="14">
+        <v>55</v>
+      </c>
+      <c r="I68" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J57" s="10" t="str">
+        <v>730</v>
+      </c>
+      <c r="J68" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K57" s="11"/>
-      <c r="L57" s="11"/>
-      <c r="M57" s="11"/>
-      <c r="N57" s="12"/>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A58" s="8"/>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="9"/>
-      <c r="F58" s="9"/>
-      <c r="G58" s="9"/>
-      <c r="H58" s="9"/>
-      <c r="I58" s="10" t="str">
+        <v>710</v>
+      </c>
+      <c r="K68" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L68" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="M68" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N68" s="16" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A69" s="13">
+        <v>46310</v>
+      </c>
+      <c r="B69" s="14">
+        <v>450</v>
+      </c>
+      <c r="C69" s="14">
+        <v>30</v>
+      </c>
+      <c r="D69" s="14">
+        <v>320</v>
+      </c>
+      <c r="E69" s="14">
+        <v>30</v>
+      </c>
+      <c r="F69" s="14">
+        <v>0</v>
+      </c>
+      <c r="G69" s="14">
+        <v>0</v>
+      </c>
+      <c r="H69" s="14">
+        <v>20</v>
+      </c>
+      <c r="I69" s="15">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J58" s="10" t="str">
+        <v>850</v>
+      </c>
+      <c r="J69" s="15">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K58" s="11"/>
-      <c r="L58" s="11"/>
-      <c r="M58" s="11"/>
-      <c r="N58" s="12"/>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A59" s="8"/>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="9"/>
-      <c r="I59" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J59" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K59" s="11"/>
-      <c r="L59" s="11"/>
-      <c r="M59" s="11"/>
-      <c r="N59" s="12"/>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A60" s="8"/>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9"/>
-      <c r="G60" s="9"/>
-      <c r="H60" s="9"/>
-      <c r="I60" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J60" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K60" s="11"/>
-      <c r="L60" s="11"/>
-      <c r="M60" s="11"/>
-      <c r="N60" s="12"/>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="8"/>
-      <c r="B61" s="9"/>
-      <c r="C61" s="9"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
-      <c r="F61" s="9"/>
-      <c r="G61" s="9"/>
-      <c r="H61" s="9"/>
-      <c r="I61" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J61" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K61" s="11"/>
-      <c r="L61" s="11"/>
-      <c r="M61" s="11"/>
-      <c r="N61" s="12"/>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="8"/>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="9"/>
-      <c r="F62" s="9"/>
-      <c r="G62" s="9"/>
-      <c r="H62" s="9"/>
-      <c r="I62" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J62" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K62" s="11"/>
-      <c r="L62" s="11"/>
-      <c r="M62" s="11"/>
-      <c r="N62" s="12"/>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="8"/>
-      <c r="B63" s="9"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="9"/>
-      <c r="F63" s="9"/>
-      <c r="G63" s="9"/>
-      <c r="H63" s="9"/>
-      <c r="I63" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J63" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K63" s="11"/>
-      <c r="L63" s="11"/>
-      <c r="M63" s="11"/>
-      <c r="N63" s="12"/>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A64" s="8"/>
-      <c r="B64" s="9"/>
-      <c r="C64" s="9"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="9"/>
-      <c r="F64" s="9"/>
-      <c r="G64" s="9"/>
-      <c r="H64" s="9"/>
-      <c r="I64" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J64" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K64" s="11"/>
-      <c r="L64" s="11"/>
-      <c r="M64" s="11"/>
-      <c r="N64" s="12"/>
-    </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A65" s="8"/>
-      <c r="B65" s="9"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="9"/>
-      <c r="F65" s="9"/>
-      <c r="G65" s="9"/>
-      <c r="H65" s="9"/>
-      <c r="I65" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J65" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K65" s="11"/>
-      <c r="L65" s="11"/>
-      <c r="M65" s="11"/>
-      <c r="N65" s="12"/>
-    </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A66" s="8"/>
-      <c r="B66" s="9"/>
-      <c r="C66" s="9"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="9"/>
-      <c r="F66" s="9"/>
-      <c r="G66" s="9"/>
-      <c r="H66" s="9"/>
-      <c r="I66" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J66" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K66" s="11"/>
-      <c r="L66" s="11"/>
-      <c r="M66" s="11"/>
-      <c r="N66" s="12"/>
-    </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A67" s="8"/>
-      <c r="B67" s="9"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="9"/>
-      <c r="F67" s="9"/>
-      <c r="G67" s="9"/>
-      <c r="H67" s="9"/>
-      <c r="I67" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J67" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K67" s="11"/>
-      <c r="L67" s="11"/>
-      <c r="M67" s="11"/>
-      <c r="N67" s="12"/>
-    </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A68" s="8"/>
-      <c r="B68" s="9"/>
-      <c r="C68" s="9"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="9"/>
-      <c r="F68" s="9"/>
-      <c r="G68" s="9"/>
-      <c r="H68" s="9"/>
-      <c r="I68" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J68" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K68" s="11"/>
-      <c r="L68" s="11"/>
-      <c r="M68" s="11"/>
-      <c r="N68" s="12"/>
-    </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A69" s="8"/>
-      <c r="B69" s="9"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="9"/>
-      <c r="F69" s="9"/>
-      <c r="G69" s="9"/>
-      <c r="H69" s="9"/>
-      <c r="I69" s="10" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J69" s="10" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="K69" s="11"/>
-      <c r="L69" s="11"/>
-      <c r="M69" s="11"/>
-      <c r="N69" s="12"/>
-    </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A70" s="8"/>
-      <c r="B70" s="9"/>
-      <c r="C70" s="9"/>
-      <c r="D70" s="9"/>
-      <c r="E70" s="9"/>
-      <c r="F70" s="9"/>
-      <c r="G70" s="9"/>
-      <c r="H70" s="9"/>
-      <c r="I70" s="10" t="str">
+        <v>590</v>
+      </c>
+      <c r="K69" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L69" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M69" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N69" s="16" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A70" s="13">
+        <v>46311</v>
+      </c>
+      <c r="B70" s="14">
+        <v>370</v>
+      </c>
+      <c r="C70" s="14">
+        <v>10</v>
+      </c>
+      <c r="D70" s="14">
+        <v>350</v>
+      </c>
+      <c r="E70" s="14">
+        <v>60</v>
+      </c>
+      <c r="F70" s="14">
+        <v>0</v>
+      </c>
+      <c r="G70" s="14">
+        <v>0</v>
+      </c>
+      <c r="H70" s="14">
+        <v>50</v>
+      </c>
+      <c r="I70" s="15">
         <f t="shared" ref="I70:I133" si="4">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
-        <v/>
-      </c>
-      <c r="J70" s="10" t="str">
+        <v>840</v>
+      </c>
+      <c r="J70" s="15">
         <f t="shared" ref="J70:J133" si="5">IF(I70="","",1440-I70)</f>
-        <v/>
-      </c>
-      <c r="K70" s="11"/>
-      <c r="L70" s="11"/>
-      <c r="M70" s="11"/>
-      <c r="N70" s="12"/>
-    </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A71" s="8"/>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="9"/>
-      <c r="F71" s="9"/>
-      <c r="G71" s="9"/>
-      <c r="H71" s="9"/>
-      <c r="I71" s="10" t="str">
+        <v>600</v>
+      </c>
+      <c r="K70" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L70" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M70" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N70" s="16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A71" s="13">
+        <v>46312</v>
+      </c>
+      <c r="B71" s="14">
+        <v>420</v>
+      </c>
+      <c r="C71" s="14">
+        <v>20</v>
+      </c>
+      <c r="D71" s="14">
+        <v>310</v>
+      </c>
+      <c r="E71" s="14">
+        <v>60</v>
+      </c>
+      <c r="F71" s="14">
+        <v>0</v>
+      </c>
+      <c r="G71" s="14">
+        <v>0</v>
+      </c>
+      <c r="H71" s="14">
+        <v>80</v>
+      </c>
+      <c r="I71" s="15">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J71" s="10" t="str">
+        <v>890</v>
+      </c>
+      <c r="J71" s="15">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K71" s="11"/>
-      <c r="L71" s="11"/>
-      <c r="M71" s="11"/>
-      <c r="N71" s="12"/>
-    </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A72" s="8"/>
-      <c r="B72" s="9"/>
-      <c r="C72" s="9"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="9"/>
-      <c r="F72" s="9"/>
-      <c r="G72" s="9"/>
-      <c r="H72" s="9"/>
-      <c r="I72" s="10" t="str">
+        <v>550</v>
+      </c>
+      <c r="K71" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L71" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M71" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N71" s="16" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A72" s="13">
+        <v>46313</v>
+      </c>
+      <c r="B72" s="14">
+        <v>510</v>
+      </c>
+      <c r="C72" s="14">
+        <v>30</v>
+      </c>
+      <c r="D72" s="14">
+        <v>20</v>
+      </c>
+      <c r="E72" s="14">
+        <v>50</v>
+      </c>
+      <c r="F72" s="14">
+        <v>0</v>
+      </c>
+      <c r="G72" s="14">
+        <v>0</v>
+      </c>
+      <c r="H72" s="14">
+        <v>240</v>
+      </c>
+      <c r="I72" s="15">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J72" s="10" t="str">
+        <v>850</v>
+      </c>
+      <c r="J72" s="15">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K72" s="11"/>
-      <c r="L72" s="11"/>
-      <c r="M72" s="11"/>
-      <c r="N72" s="12"/>
-    </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A73" s="8"/>
-      <c r="B73" s="9"/>
-      <c r="C73" s="9"/>
-      <c r="D73" s="9"/>
-      <c r="E73" s="9"/>
-      <c r="F73" s="9"/>
-      <c r="G73" s="9"/>
-      <c r="H73" s="9"/>
-      <c r="I73" s="10" t="str">
+        <v>590</v>
+      </c>
+      <c r="K72" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L72" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M72" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N72" s="16" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A73" s="13">
+        <v>46314</v>
+      </c>
+      <c r="B73" s="14">
+        <v>390</v>
+      </c>
+      <c r="C73" s="14">
+        <v>20</v>
+      </c>
+      <c r="D73" s="14">
+        <v>50</v>
+      </c>
+      <c r="E73" s="14">
+        <v>60</v>
+      </c>
+      <c r="F73" s="14">
+        <v>200</v>
+      </c>
+      <c r="G73" s="14">
+        <v>4</v>
+      </c>
+      <c r="H73" s="14">
+        <v>60</v>
+      </c>
+      <c r="I73" s="15">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J73" s="10" t="str">
+        <v>780</v>
+      </c>
+      <c r="J73" s="15">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K73" s="11"/>
-      <c r="L73" s="11"/>
-      <c r="M73" s="11"/>
-      <c r="N73" s="12"/>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A74" s="8"/>
-      <c r="B74" s="9"/>
-      <c r="C74" s="9"/>
-      <c r="D74" s="9"/>
-      <c r="E74" s="9"/>
-      <c r="F74" s="9"/>
-      <c r="G74" s="9"/>
-      <c r="H74" s="9"/>
-      <c r="I74" s="10" t="str">
+        <v>660</v>
+      </c>
+      <c r="K73" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L73" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M73" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N73" s="16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A74" s="13">
+        <v>46315</v>
+      </c>
+      <c r="B74" s="14">
+        <v>490</v>
+      </c>
+      <c r="C74" s="14">
+        <v>30</v>
+      </c>
+      <c r="D74" s="14">
+        <v>60</v>
+      </c>
+      <c r="E74" s="14">
+        <v>80</v>
+      </c>
+      <c r="F74" s="14">
+        <v>0</v>
+      </c>
+      <c r="G74" s="14">
+        <v>0</v>
+      </c>
+      <c r="H74" s="14">
+        <v>180</v>
+      </c>
+      <c r="I74" s="15">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J74" s="10" t="str">
+        <v>840</v>
+      </c>
+      <c r="J74" s="15">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K74" s="11"/>
-      <c r="L74" s="11"/>
-      <c r="M74" s="11"/>
-      <c r="N74" s="12"/>
-    </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A75" s="8"/>
-      <c r="B75" s="9"/>
-      <c r="C75" s="9"/>
-      <c r="D75" s="9"/>
-      <c r="E75" s="9"/>
-      <c r="F75" s="9"/>
-      <c r="G75" s="9"/>
-      <c r="H75" s="9"/>
-      <c r="I75" s="10" t="str">
+        <v>600</v>
+      </c>
+      <c r="K74" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L74" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M74" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N74" s="16" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A75" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B75" s="14">
+        <v>450</v>
+      </c>
+      <c r="C75" s="14">
+        <v>20</v>
+      </c>
+      <c r="D75" s="14">
+        <v>50</v>
+      </c>
+      <c r="E75" s="14">
+        <v>40</v>
+      </c>
+      <c r="F75" s="14">
+        <v>250</v>
+      </c>
+      <c r="G75" s="14">
+        <v>5</v>
+      </c>
+      <c r="H75" s="14">
+        <v>80</v>
+      </c>
+      <c r="I75" s="15">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="J75" s="10" t="str">
+        <v>890</v>
+      </c>
+      <c r="J75" s="15">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="K75" s="11"/>
-      <c r="L75" s="11"/>
-      <c r="M75" s="11"/>
-      <c r="N75" s="12"/>
+        <v>550</v>
+      </c>
+      <c r="K75" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L75" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M75" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N75" s="16" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" s="8"/>

</xml_diff>